<commit_message>
feat: compatible with flowcell 2 data
</commit_message>
<xml_diff>
--- a/data/input/custom_feature_annotations.xlsx
+++ b/data/input/custom_feature_annotations.xlsx
@@ -433,7 +433,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z23"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.88"/>
   </cols>
@@ -783,11 +783,11 @@
   <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="17.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="6" width="14.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="6" width="14.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="6" width="18.24"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="12.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="6" width="10.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="6" width="6.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="6" width="8.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="6" width="17.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="6" width="18.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="6" width="16.02"/>
@@ -1071,7 +1071,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
   </cols>

</xml_diff>

<commit_message>
feat: rDNA coverage table and other figure updates
</commit_message>
<xml_diff>
--- a/data/input/custom_feature_annotations.xlsx
+++ b/data/input/custom_feature_annotations.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="filtering" sheetId="1" state="visible" r:id="rId2"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="70">
   <si>
     <t xml:space="preserve">Feature</t>
   </si>
@@ -162,9 +162,6 @@
   </si>
   <si>
     <t xml:space="preserve">pseudogene</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anti-feature</t>
   </si>
   <si>
     <t xml:space="preserve">RNA.Polymerase</t>
@@ -771,12 +768,8 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0"/>
@@ -823,16 +816,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>41</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>42</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>2</v>
@@ -847,13 +840,13 @@
         <v>4</v>
       </c>
       <c r="I1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>45</v>
       </c>
       <c r="L1" s="9"/>
       <c r="M1" s="9"/>
@@ -879,16 +872,16 @@
         <v>3</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="10" t="s">
         <v>48</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>9</v>
@@ -905,7 +898,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -913,16 +906,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>53</v>
-      </c>
       <c r="E4" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>9</v>
@@ -939,13 +932,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>54</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>55</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>16</v>
@@ -965,13 +958,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>16</v>
@@ -991,13 +984,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>59</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>16</v>
@@ -1017,16 +1010,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="E8" s="10" t="s">
         <v>61</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>62</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>21</v>
@@ -1043,16 +1036,16 @@
         <v>3</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>64</v>
-      </c>
       <c r="E9" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>9</v>
@@ -1069,13 +1062,13 @@
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="J10" s="7" t="s">
         <v>65</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>66</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>500</v>
@@ -1101,29 +1094,29 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.7421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>